<commit_message>
Demo sin nombres ni códigos de aerolínea reales
Empleados con código (EMP001…) y vuelos XX con números inventados, también
en los ejemplos y en las pruebas. Noviembre de la demo: programa 12.587 h y
6 h sin cubrir; a mano 14.057 h y 520 h.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JKUiQJ7u1SQbQddix7SeeH
</commit_message>
<xml_diff>
--- a/ejemplos/demo/contratos.xlsx
+++ b/ejemplos/demo/contratos.xlsx
@@ -431,7 +431,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>FUENTES LOZANO, ELENA</t>
+          <t>EMP001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -443,115 +443,115 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ALONSO ALONSO, MARTA</t>
+          <t>EMP002</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>TCC</t>
+          <t>TC</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>DELGADO MOLINA, YOLANDA</t>
+          <t>EMP003</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>EVE</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>DELGADO PEÑA, YOLANDA</t>
+          <t>EMP004</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>TC</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>FUENTES PEÑA, ÓSCAR</t>
+          <t>EMP005</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>EVE</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ALONSO CANO, ALBA</t>
+          <t>EMP006</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>GALLEGO CASTRO, PABLO</t>
+          <t>EMP007</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>TC</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>BLANCO SANTOS, MIGUEL</t>
+          <t>EMP008</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>GARRIDO ALONSO, ADRIÁN</t>
+          <t>EMP009</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>TC</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>GALLEGO VEGA, YOLANDA</t>
+          <t>EMP010</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>TC</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>DÍAZ LEÓN, CARLOS</t>
+          <t>EMP011</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -563,31 +563,31 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>DELGADO MÉNDEZ, ÓSCAR</t>
+          <t>EMP012</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>TCC</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CASTRO HERRERA, VALERIA</t>
+          <t>EMP013</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>FUENTES HERRERA, VALERIA</t>
+          <t>EMP014</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -599,7 +599,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CASTRO MÉNDEZ, ALBA</t>
+          <t>EMP015</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -611,7 +611,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ALONSO IGLESIAS, RAÚL</t>
+          <t>EMP016</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -623,19 +623,19 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>DÍAZ BLANCO, PAULA</t>
+          <t>EMP017</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>FD</t>
+          <t>EVE</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>CANO LOZANO, FERNANDO</t>
+          <t>EMP018</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -647,7 +647,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>ALONSO VEGA, ROCÍO</t>
+          <t>EMP019</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -659,19 +659,19 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ALONSO PASTOR, ANA</t>
+          <t>EMP020</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>FD</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>CASTRO PEÑA, ROCÍO</t>
+          <t>EMP021</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -683,31 +683,31 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>CASTRO IGLESIAS, MARTA</t>
+          <t>EMP022</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>BLANCO MÉNDEZ, VÍCTOR</t>
+          <t>EMP023</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>TCC</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>DELGADO SOTO, ADRIÁN</t>
+          <t>EMP024</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -719,7 +719,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>CASTRO VIDAL, DANIEL</t>
+          <t>EMP025</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -731,31 +731,31 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>DELGADO SERRANO, TOMÁS</t>
+          <t>EMP026</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>TC</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>ALONSO CASTRO, LAURA</t>
+          <t>EMP027</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>FD</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>HERRERA CANO, LUIS</t>
+          <t>EMP028</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -767,7 +767,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>GARRIDO MÉNDEZ, MANUEL</t>
+          <t>EMP029</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -779,55 +779,55 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>LEÓN CASTRO, CLAUDIA</t>
+          <t>EMP030</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>TC</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>HERRERA MÉNDEZ, CARMEN</t>
+          <t>EMP031</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>FD</t>
+          <t>TC</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>IGLESIAS MORALES, MANUEL</t>
+          <t>EMP032</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>FD</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>GARRIDO SOTO, ANDRÉS</t>
+          <t>EMP033</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>GARRIDO PRIETO, SARA</t>
+          <t>EMP034</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -839,67 +839,67 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>GARRIDO RAMOS, MANUEL</t>
+          <t>EMP035</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>HERRERA MÉNDEZ, IRENE</t>
+          <t>EMP036</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>EVE</t>
+          <t>TC</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>HERRERA MÉNDEZ, CARLOS</t>
+          <t>EMP037</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>EVE</t>
+          <t>TC</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>GARRIDO VIDAL, MANUEL</t>
+          <t>EMP038</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>FD</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>GARRIDO NAVARRO, LAURA</t>
+          <t>EMP039</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>HERRERA IGLESIAS, LUCÍA</t>
+          <t>EMP040</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -911,67 +911,67 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>LEÓN ZAMORA, SARA</t>
+          <t>EMP041</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>LEÓN ZAMORA, JAVIER</t>
+          <t>EMP042</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>MARÍN NAVARRO, RAÚL</t>
+          <t>EMP043</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>TC</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>MARÍN MORALES, TOMÁS</t>
+          <t>EMP044</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>EVE</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>LEÓN LEÓN, LUCÍA</t>
+          <t>EMP045</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>MARÍN SOTO, SERGIO</t>
+          <t>EMP046</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -983,55 +983,55 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>LOZANO GARRIDO, LUIS</t>
+          <t>EMP047</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>TC</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>LEÓN ZAMORA, CLAUDIA</t>
+          <t>EMP048</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>MARÍN PASTOR, IRENE</t>
+          <t>EMP049</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>TC</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>MARÍN CANO, LAURA</t>
+          <t>EMP050</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>TC</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>MOLINA IGLESIAS, RAÚL</t>
+          <t>EMP051</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1043,7 +1043,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>MOLINA PRIETO, IRENE</t>
+          <t>EMP052</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -1055,19 +1055,19 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>MOLINA RAMOS, RAÚL</t>
+          <t>EMP053</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>FD</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>MOLINA CANO, PAULA</t>
+          <t>EMP054</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1079,19 +1079,19 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>MOLINA VEGA, ANDRÉS</t>
+          <t>EMP055</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>TCC</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>ORTEGA ORTEGA, SARA</t>
+          <t>EMP056</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -1103,31 +1103,31 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>NAVARRO LOZANO, ADRIÁN</t>
+          <t>EMP057</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>PASTOR MÉNDEZ, TOMÁS</t>
+          <t>EMP058</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>EVE</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>PEÑA LEÓN, CARMEN</t>
+          <t>EMP059</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -1139,7 +1139,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>MÉNDEZ PASTOR, DANIEL</t>
+          <t>EMP060</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -1151,19 +1151,19 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>RAMOS MORALES, YOLANDA</t>
+          <t>EMP061</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>FD</t>
+          <t>TC</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>SERRANO MORALES, ELENA</t>
+          <t>EMP062</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1175,19 +1175,19 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>SERRANO DELGADO, MARTA</t>
+          <t>EMP063</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>TC</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>PRIETO VEGA, CARLOS</t>
+          <t>EMP064</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1199,7 +1199,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>MORALES MARÍN, LAURA</t>
+          <t>EMP065</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1211,7 +1211,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>RAMOS MOLINA, TOMÁS</t>
+          <t>EMP066</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -1223,19 +1223,19 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>SERRANO LOZANO, SERGIO</t>
+          <t>EMP067</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>FD</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>SERRANO VIDAL, MARTA</t>
+          <t>EMP068</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -1247,7 +1247,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>NAVARRO ZAMORA, VALERIA</t>
+          <t>EMP069</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -1259,19 +1259,19 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>MORALES ZAMORA, MANUEL</t>
+          <t>EMP070</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>RAMOS RUBIO, CARMEN</t>
+          <t>EMP071</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -1283,31 +1283,31 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>MÉNDEZ PRIETO, MANUEL</t>
+          <t>EMP072</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>PRIETO CASTRO, ROCÍO</t>
+          <t>EMP073</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>EVE</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>RUBIO VEGA, LUIS</t>
+          <t>EMP074</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -1319,55 +1319,55 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>SANTOS PEÑA, CLAUDIA</t>
+          <t>EMP075</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>FD</t>
+          <t>TC</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>MÉNDEZ ORTEGA, MIGUEL</t>
+          <t>EMP076</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>SERRANO PEÑA, MARTA</t>
+          <t>EMP077</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>EVE</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>MÉNDEZ ORTEGA, PABLO</t>
+          <t>EMP078</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>MÉNDEZ ZAMORA, CARLOS</t>
+          <t>EMP079</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -1379,31 +1379,31 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>MOLINA SANTOS, SARA</t>
+          <t>EMP080</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>ORTEGA NAVARRO, VALERIA</t>
+          <t>EMP081</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>EVE</t>
+          <t>TC</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>PRIETO HERRERA, MIGUEL</t>
+          <t>EMP082</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -1415,19 +1415,19 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>ORTEGA GALLEGO, SARA</t>
+          <t>EMP083</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>EVE</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>SERRANO DÍAZ, CARMEN</t>
+          <t>EMP084</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -1439,43 +1439,43 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>PASTOR SERRANO, CLAUDIA</t>
+          <t>EMP085</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>TC</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>RUBIO SANTOS, SARA</t>
+          <t>EMP086</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>TCC</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>MÉNDEZ CASTRO, MARTA</t>
+          <t>EMP087</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>ORTEGA MÉNDEZ, DANIEL</t>
+          <t>EMP088</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -1487,67 +1487,67 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>NAVARRO NAVARRO, FERNANDO</t>
+          <t>EMP089</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>EVE</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>NAVARRO MARÍN, VÍCTOR</t>
+          <t>EMP090</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>FD</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>MORALES PEÑA, ANA</t>
+          <t>EMP091</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>EVE</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>RAMOS ZAMORA, MIGUEL</t>
+          <t>EMP092</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>EVE</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>SERRANO FUENTES, LAURA</t>
+          <t>EMP093</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>TC</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>MÉNDEZ RAMOS, ROCÍO</t>
+          <t>EMP094</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -1559,7 +1559,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>NAVARRO GALLEGO, MANUEL</t>
+          <t>EMP095</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -1571,31 +1571,31 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>SANTOS SOTO, LUIS</t>
+          <t>EMP096</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>FD</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>MORALES SERRANO, ALBA</t>
+          <t>EMP097</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>PRIETO DÍAZ, ÓSCAR</t>
+          <t>EMP098</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -1607,19 +1607,19 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>RUBIO IGLESIAS, ANA</t>
+          <t>EMP099</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>TC</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>PEÑA MORALES, CLAUDIA</t>
+          <t>EMP100</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -1631,7 +1631,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>PRIETO RAMOS, ANA</t>
+          <t>EMP101</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -1643,19 +1643,19 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>ORTEGA DELGADO, PABLO</t>
+          <t>EMP102</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>TC</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>PASTOR MARÍN, MANUEL</t>
+          <t>EMP103</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -1667,31 +1667,31 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>ORTEGA MORALES, CLAUDIA</t>
+          <t>EMP104</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>TC</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>MORALES PEÑA, VÍCTOR</t>
+          <t>EMP105</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>NAVARRO MARÍN, TOMÁS</t>
+          <t>EMP106</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -1703,19 +1703,19 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>MÉNDEZ MORALES, SARA</t>
+          <t>EMP107</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>SERRANO MORALES, TOMÁS</t>
+          <t>EMP108</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -1727,55 +1727,55 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>SANTOS VEGA, PABLO</t>
+          <t>EMP109</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>TC</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>RAMOS ORTEGA, FERNANDO</t>
+          <t>EMP110</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>TC</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>SOTO MOLINA, TOMÁS</t>
+          <t>EMP111</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>FD</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>SOTO VIDAL, RAÚL</t>
+          <t>EMP112</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>TC</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>VIDAL ALONSO, CARMEN</t>
+          <t>EMP113</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -1787,31 +1787,31 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>VEGA MARÍN, NEREA</t>
+          <t>EMP114</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>TC</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>SOTO LEÓN, PAULA</t>
+          <t>EMP115</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>VEGA FUENTES, DANIEL</t>
+          <t>EMP116</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -1823,31 +1823,31 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>VIDAL LOZANO, LUIS</t>
+          <t>EMP117</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>VIDAL CANO, ADRIÁN</t>
+          <t>EMP118</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>VIDAL PASTOR, PABLO</t>
+          <t>EMP119</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -1859,19 +1859,19 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>VIDAL ORTEGA, MIGUEL</t>
+          <t>EMP120</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>TC</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>VIDAL MOLINA, LAURA</t>
+          <t>EMP121</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -1883,43 +1883,43 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>VIDAL RAMOS, MARTA</t>
+          <t>EMP122</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>TC</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>VIDAL DELGADO, CARLOS</t>
+          <t>EMP123</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>VIDAL PEÑA, ROCÍO</t>
+          <t>EMP124</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>TC</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>ZAMORA VEGA, MANUEL</t>
+          <t>EMP125</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -1931,7 +1931,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>ZAMORA CASTRO, MANUEL</t>
+          <t>EMP126</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -1943,7 +1943,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>ZAMORA ORTEGA, FERNANDO</t>
+          <t>EMP127</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -1955,7 +1955,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>ZAMORA MOLINA, MARTA</t>
+          <t>EMP128</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -1967,7 +1967,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>ZAMORA BLANCO, VALERIA</t>
+          <t>EMP129</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -1979,7 +1979,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>ZAMORA SERRANO, ANDRÉS</t>
+          <t>EMP130</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -1991,7 +1991,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>ZAMORA MORALES, ELENA</t>
+          <t>EMP131</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -2003,7 +2003,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>ZAMORA SOTO, ANA</t>
+          <t>EMP132</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">

</xml_diff>

<commit_message>
Pasaje: facturación, embarque, puestos fijos y responsables
- pasaje en la configuración (desactivado en el perfil de Azul): 4 personas
  por facturación, 2 por embarque, oficina 2, lost and found 1 y un
  responsable a la vez durante la operación.
- El cuadrante del mes y el resumen planifican también Pasaje y Responsable
  pasaje. La parrilla del día añade la hoja Pasaje con quién factura y
  embarca cada vuelo y quién está en los puestos fijos, con relevos.
- Configuración por herencia (hereda: base.yaml); config/demo.yaml activa
  pasaje y la web lo usa en modo demo. La demo tiene 125 agentes y 3
  responsables de pasaje.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JKUiQJ7u1SQbQddix7SeeH
</commit_message>
<xml_diff>
--- a/ejemplos/demo/contratos.xlsx
+++ b/ejemplos/demo/contratos.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B133"/>
+  <dimension ref="A1:B261"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,7 +436,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>TC</t>
         </is>
       </c>
     </row>
@@ -460,7 +460,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>EVE</t>
+          <t>TC</t>
         </is>
       </c>
     </row>
@@ -484,7 +484,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>TC</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>EVE</t>
         </is>
       </c>
     </row>
@@ -520,7 +520,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>TCC</t>
         </is>
       </c>
     </row>
@@ -532,7 +532,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
@@ -544,7 +544,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
@@ -556,7 +556,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>TC</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>TCC</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
@@ -592,7 +592,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>TC</t>
         </is>
       </c>
     </row>
@@ -604,7 +604,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
@@ -628,7 +628,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>EVE</t>
+          <t>FD</t>
         </is>
       </c>
     </row>
@@ -652,7 +652,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
@@ -664,7 +664,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>FD</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>FD</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>EVE</t>
         </is>
       </c>
     </row>
@@ -700,7 +700,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>TCC</t>
+          <t>TC</t>
         </is>
       </c>
     </row>
@@ -724,7 +724,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
@@ -736,7 +736,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>TCC</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>FD</t>
+          <t>TC</t>
         </is>
       </c>
     </row>
@@ -784,7 +784,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>FD</t>
         </is>
       </c>
     </row>
@@ -820,7 +820,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>TC</t>
         </is>
       </c>
     </row>
@@ -832,7 +832,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
@@ -856,7 +856,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
@@ -868,7 +868,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
@@ -880,7 +880,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>FD</t>
+          <t>TC</t>
         </is>
       </c>
     </row>
@@ -892,7 +892,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>TC</t>
         </is>
       </c>
     </row>
@@ -904,7 +904,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>TC</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>TC</t>
         </is>
       </c>
     </row>
@@ -976,7 +976,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>TC</t>
         </is>
       </c>
     </row>
@@ -988,7 +988,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
@@ -1048,7 +1048,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>TC</t>
         </is>
       </c>
     </row>
@@ -1072,7 +1072,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
@@ -1084,7 +1084,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>TC</t>
         </is>
       </c>
     </row>
@@ -1120,7 +1120,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>EVE</t>
+          <t>TC</t>
         </is>
       </c>
     </row>
@@ -1132,7 +1132,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>TC</t>
         </is>
       </c>
     </row>
@@ -1156,7 +1156,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
@@ -1180,7 +1180,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
@@ -1228,7 +1228,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>FD</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
@@ -1240,7 +1240,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>TC</t>
         </is>
       </c>
     </row>
@@ -1276,7 +1276,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>EVE</t>
         </is>
       </c>
     </row>
@@ -1288,7 +1288,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>EVE</t>
         </is>
       </c>
     </row>
@@ -1324,7 +1324,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
@@ -1336,7 +1336,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>TC</t>
         </is>
       </c>
     </row>
@@ -1348,7 +1348,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>EVE</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
@@ -1372,7 +1372,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>EVE</t>
         </is>
       </c>
     </row>
@@ -1384,7 +1384,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>EVE</t>
         </is>
       </c>
     </row>
@@ -1420,7 +1420,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>EVE</t>
+          <t>TC</t>
         </is>
       </c>
     </row>
@@ -1432,7 +1432,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>TC</t>
         </is>
       </c>
     </row>
@@ -1456,7 +1456,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>TCC</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
@@ -1468,7 +1468,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>TC</t>
         </is>
       </c>
     </row>
@@ -1480,7 +1480,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>TC</t>
         </is>
       </c>
     </row>
@@ -1492,7 +1492,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>EVE</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
@@ -1504,7 +1504,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>FD</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
@@ -1516,7 +1516,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>EVE</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
@@ -1528,7 +1528,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>EVE</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
@@ -1540,7 +1540,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
@@ -1552,7 +1552,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>EVE</t>
         </is>
       </c>
     </row>
@@ -1564,7 +1564,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
@@ -1600,7 +1600,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>FD</t>
         </is>
       </c>
     </row>
@@ -1612,7 +1612,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
@@ -1624,7 +1624,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>TC</t>
         </is>
       </c>
     </row>
@@ -1636,7 +1636,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>TCC</t>
         </is>
       </c>
     </row>
@@ -1648,7 +1648,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
@@ -1684,7 +1684,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>FD</t>
         </is>
       </c>
     </row>
@@ -1720,7 +1720,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>TC</t>
         </is>
       </c>
     </row>
@@ -1732,7 +1732,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
@@ -1744,7 +1744,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>EVE</t>
         </is>
       </c>
     </row>
@@ -1756,7 +1756,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>FD</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
@@ -1780,7 +1780,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>FD</t>
         </is>
       </c>
     </row>
@@ -1792,7 +1792,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
@@ -1804,7 +1804,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>TC</t>
         </is>
       </c>
     </row>
@@ -1876,7 +1876,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>TC</t>
         </is>
       </c>
     </row>
@@ -1888,7 +1888,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
@@ -1900,7 +1900,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>TC</t>
         </is>
       </c>
     </row>
@@ -1912,7 +1912,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
@@ -1924,7 +1924,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
@@ -1960,7 +1960,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
@@ -1972,7 +1972,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
@@ -1984,7 +1984,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
@@ -1996,7 +1996,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>TC</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
@@ -2007,6 +2007,1542 @@
         </is>
       </c>
       <c r="B133" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>EMP133</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>TC</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>EMP134</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>EMP135</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>EMP136</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>EMP137</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>EMP138</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>EMP139</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>TC</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>EMP140</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>FD</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>EMP141</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>TC</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>EMP142</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>EMP143</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>EMP144</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>TC</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>EMP145</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>TC</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>EMP146</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>EMP147</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>EMP148</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>EMP149</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>EMP150</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>EMP151</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>TC</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>EMP152</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>TC</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>EMP153</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>EVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>EMP154</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>EMP155</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>EMP156</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>EMP157</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>EMP158</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>EMP159</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>EMP160</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>FD</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>EMP161</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>TCC</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>EMP162</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>EMP163</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>EMP164</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>TC</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>EMP165</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>EMP166</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>TC</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>EMP167</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>EMP168</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>EMP169</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>EMP170</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>FD</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>EMP171</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>EMP172</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>EMP173</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>TC</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>EMP174</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>TC</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>EMP175</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>EMP176</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>EMP177</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>TC</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>EMP178</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>EMP179</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>EMP180</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>TC</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>EMP181</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>EMP182</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>TC</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>EMP183</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>TC</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>EMP184</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>EMP185</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>TCC</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>EMP186</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>EMP187</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>EMP188</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>EMP189</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>EMP190</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>EMP191</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>TCC</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>EMP192</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>EVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>EMP193</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>TC</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>EMP194</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>EMP195</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>EVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>EMP196</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>EMP197</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>EMP198</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>EMP199</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>TC</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>EMP200</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>EMP201</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>FD</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>EMP202</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>EMP203</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>TC</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>EMP204</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>EMP205</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>EMP206</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>EMP207</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>EMP208</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>EMP209</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>EMP210</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>TC</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>EMP211</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>TC</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>EMP212</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>EMP213</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>EVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>EMP214</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>EVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>EMP215</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>EMP216</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>EMP217</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>EVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>EMP218</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>EMP219</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>EMP220</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>EMP221</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>TC</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>EMP222</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>TC</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>EMP223</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>FD</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>EMP224</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>TC</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>EMP225</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>EMP226</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>TC</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>EMP227</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>EMP228</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>TC</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>EMP229</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>EMP230</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>TC</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>EMP231</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>TC</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>EMP232</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>EMP233</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>EMP234</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>EMP235</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>EMP236</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>TC</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>EMP237</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>TC</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>EMP238</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>EMP239</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>EMP240</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>EMP241</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>EMP242</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>TC</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>EMP243</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>TC</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>EMP244</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>EMP245</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>EMP246</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>EMP247</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>TC</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>EMP248</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>EMP249</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>TC</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>EMP250</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>TCC</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>EMP251</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>TC</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>EMP252</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>TC</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>EMP253</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>TC</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>EMP254</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>TC</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>EMP255</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>TC</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>EMP256</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>TC</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>EMP257</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>TC</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>EMP258</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>TCC</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>EMP259</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>TCC</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>EMP260</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
         <is>
           <t>TC</t>
         </is>

</xml_diff>